<commit_message>
TestNG, reflections, POM, PageFactory
</commit_message>
<xml_diff>
--- a/Runner/RunController.xlsx
+++ b/Runner/RunController.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TESTING\Selenium_Workspace\Runner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A489A559-3626-482E-8949-1B5BA049B588}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB7B921-C6FD-4ECD-9D03-F9B449EF4058}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -452,7 +452,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -518,7 +518,7 @@
         <v>14</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>